<commit_message>
chore: update Fanqie male rankings
</commit_message>
<xml_diff>
--- a/data/持续收益潜力作品.xlsx
+++ b/data/持续收益潜力作品.xlsx
@@ -10,19 +10,19 @@
     <sheet name="作品数据" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">作品数据!$A$4:$O$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">作品数据!$A$4:$O$12</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="26">
   <si>
     <t>持续收益潜力作品</t>
   </si>
   <si>
-    <t>生成时间：—。候选名单仅依据公开榜单的连续出现、在读规模和在读变化筛选，不代表真实稿费、订阅收入或平台结算。</t>
+    <t>生成时间：2026-07-25T07:38:52+00:00。候选名单仅依据公开榜单的连续出现、在读规模和在读变化筛选，不代表真实稿费、订阅收入或平台结算。</t>
   </si>
   <si>
     <t>作品名</t>
@@ -68,13 +68,44 @@
   </si>
   <si>
     <t>达标日期列表</t>
+  </si>
+  <si>
+    <t>穿越自带炼妖壶：桀桀，顷刻炼化</t>
+  </si>
+  <si>
+    <t>打开作品</t>
+  </si>
+  <si>
+    <t>领主：我在苦痛世界，养成少女</t>
+  </si>
+  <si>
+    <t>早知道不这么玩了！</t>
+  </si>
+  <si>
+    <t>异世界：我的人生开了挂！</t>
+  </si>
+  <si>
+    <t>什么！我们家居然是邪神后裔？</t>
+  </si>
+  <si>
+    <t>西幻：我有一本冒险者指南</t>
+  </si>
+  <si>
+    <t>从零开始的黑暗童话世界</t>
+  </si>
+  <si>
+    <t>穿越异世界，我能看见经验条</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="4">
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="#,##0.0"/>
+    <numFmt numFmtId="165" formatCode="#,##0"/>
+  </numFmts>
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -105,6 +136,14 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF0563C1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -126,7 +165,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -149,11 +188,26 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFE6E6E6"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFE6E6E6"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFE6E6E6"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFE6E6E6"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -163,6 +217,18 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -458,7 +524,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O4"/>
+  <dimension ref="A1:O12"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="28.7109375" customWidth="1"/>
@@ -561,12 +627,286 @@
         <v>16</v>
       </c>
     </row>
+    <row r="5" spans="1:15">
+      <c r="A5" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B5" s="5"/>
+      <c r="C5" s="5">
+        <v>81.3</v>
+      </c>
+      <c r="D5" s="4"/>
+      <c r="E5" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="F5" s="7">
+        <v>169000</v>
+      </c>
+      <c r="G5" s="7">
+        <v>19000</v>
+      </c>
+      <c r="H5" s="7">
+        <v>3</v>
+      </c>
+      <c r="I5" s="7">
+        <v>19000</v>
+      </c>
+      <c r="J5" s="5">
+        <v>58.5</v>
+      </c>
+      <c r="K5" s="4"/>
+      <c r="L5" s="4"/>
+      <c r="M5" s="7"/>
+      <c r="N5" s="5"/>
+      <c r="O5" s="4"/>
+    </row>
+    <row r="6" spans="1:15">
+      <c r="A6" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="B6" s="5"/>
+      <c r="C6" s="5">
+        <v>79.40000000000001</v>
+      </c>
+      <c r="D6" s="4"/>
+      <c r="E6" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="F6" s="7">
+        <v>433000</v>
+      </c>
+      <c r="G6" s="7">
+        <v>5000</v>
+      </c>
+      <c r="H6" s="7">
+        <v>3</v>
+      </c>
+      <c r="I6" s="7">
+        <v>6000</v>
+      </c>
+      <c r="J6" s="5">
+        <v>54.2</v>
+      </c>
+      <c r="K6" s="4"/>
+      <c r="L6" s="4"/>
+      <c r="M6" s="7"/>
+      <c r="N6" s="5"/>
+      <c r="O6" s="4"/>
+    </row>
+    <row r="7" spans="1:15">
+      <c r="A7" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B7" s="5"/>
+      <c r="C7" s="5">
+        <v>74.40000000000001</v>
+      </c>
+      <c r="D7" s="4"/>
+      <c r="E7" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="F7" s="7">
+        <v>191000</v>
+      </c>
+      <c r="G7" s="7">
+        <v>1000</v>
+      </c>
+      <c r="H7" s="7">
+        <v>3</v>
+      </c>
+      <c r="I7" s="7">
+        <v>500</v>
+      </c>
+      <c r="J7" s="5">
+        <v>50</v>
+      </c>
+      <c r="K7" s="4"/>
+      <c r="L7" s="4"/>
+      <c r="M7" s="7"/>
+      <c r="N7" s="5"/>
+      <c r="O7" s="4"/>
+    </row>
+    <row r="8" spans="1:15">
+      <c r="A8" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B8" s="5"/>
+      <c r="C8" s="5">
+        <v>72.90000000000001</v>
+      </c>
+      <c r="D8" s="4"/>
+      <c r="E8" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="F8" s="7">
+        <v>179000</v>
+      </c>
+      <c r="G8" s="7">
+        <v>0</v>
+      </c>
+      <c r="H8" s="7">
+        <v>3</v>
+      </c>
+      <c r="I8" s="7">
+        <v>0</v>
+      </c>
+      <c r="J8" s="5">
+        <v>49.1</v>
+      </c>
+      <c r="K8" s="4"/>
+      <c r="L8" s="4"/>
+      <c r="M8" s="7"/>
+      <c r="N8" s="5"/>
+      <c r="O8" s="4"/>
+    </row>
+    <row r="9" spans="1:15">
+      <c r="A9" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="B9" s="5"/>
+      <c r="C9" s="5">
+        <v>72.2</v>
+      </c>
+      <c r="D9" s="4"/>
+      <c r="E9" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="F9" s="7">
+        <v>152000</v>
+      </c>
+      <c r="G9" s="7">
+        <v>2000</v>
+      </c>
+      <c r="H9" s="7">
+        <v>3</v>
+      </c>
+      <c r="I9" s="7">
+        <v>1000</v>
+      </c>
+      <c r="J9" s="5">
+        <v>49</v>
+      </c>
+      <c r="K9" s="4"/>
+      <c r="L9" s="4"/>
+      <c r="M9" s="7"/>
+      <c r="N9" s="5"/>
+      <c r="O9" s="4"/>
+    </row>
+    <row r="10" spans="1:15">
+      <c r="A10" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="B10" s="5"/>
+      <c r="C10" s="5">
+        <v>71.3</v>
+      </c>
+      <c r="D10" s="4"/>
+      <c r="E10" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="F10" s="7">
+        <v>149000</v>
+      </c>
+      <c r="G10" s="7">
+        <v>3000</v>
+      </c>
+      <c r="H10" s="7">
+        <v>3</v>
+      </c>
+      <c r="I10" s="7">
+        <v>2000</v>
+      </c>
+      <c r="J10" s="5">
+        <v>48.7</v>
+      </c>
+      <c r="K10" s="4"/>
+      <c r="L10" s="4"/>
+      <c r="M10" s="7"/>
+      <c r="N10" s="5"/>
+      <c r="O10" s="4"/>
+    </row>
+    <row r="11" spans="1:15">
+      <c r="A11" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="B11" s="5"/>
+      <c r="C11" s="5">
+        <v>68.09999999999999</v>
+      </c>
+      <c r="D11" s="4"/>
+      <c r="E11" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="F11" s="7">
+        <v>124000</v>
+      </c>
+      <c r="G11" s="7">
+        <v>7000</v>
+      </c>
+      <c r="H11" s="7">
+        <v>3</v>
+      </c>
+      <c r="I11" s="7">
+        <v>3500</v>
+      </c>
+      <c r="J11" s="5">
+        <v>47.3</v>
+      </c>
+      <c r="K11" s="4"/>
+      <c r="L11" s="4"/>
+      <c r="M11" s="7"/>
+      <c r="N11" s="5"/>
+      <c r="O11" s="4"/>
+    </row>
+    <row r="12" spans="1:15">
+      <c r="A12" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="B12" s="5"/>
+      <c r="C12" s="5">
+        <v>67.09999999999999</v>
+      </c>
+      <c r="D12" s="4"/>
+      <c r="E12" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="F12" s="7">
+        <v>126000</v>
+      </c>
+      <c r="G12" s="7">
+        <v>2000</v>
+      </c>
+      <c r="H12" s="7">
+        <v>3</v>
+      </c>
+      <c r="I12" s="7">
+        <v>1000</v>
+      </c>
+      <c r="J12" s="5">
+        <v>46.2</v>
+      </c>
+      <c r="K12" s="4"/>
+      <c r="L12" s="4"/>
+      <c r="M12" s="7"/>
+      <c r="N12" s="5"/>
+      <c r="O12" s="4"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:O5"/>
+  <autoFilter ref="A4:O12"/>
   <mergeCells count="2">
     <mergeCell ref="A1:O1"/>
     <mergeCell ref="A2:O2"/>
   </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="E5" r:id="rId1"/>
+    <hyperlink ref="E6" r:id="rId2"/>
+    <hyperlink ref="E7" r:id="rId3"/>
+    <hyperlink ref="E8" r:id="rId4"/>
+    <hyperlink ref="E9" r:id="rId5"/>
+    <hyperlink ref="E10" r:id="rId6"/>
+    <hyperlink ref="E11" r:id="rId7"/>
+    <hyperlink ref="E12" r:id="rId8"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>